<commit_message>
Add image support for questions and explanations
</commit_message>
<xml_diff>
--- a/data/question_master_test_1.xlsx
+++ b/data/question_master_test_1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\km78617\Desktop\DX・AI関連\競技大会学科\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\km78617\Documents\GitHub\kikai-gakka-exam\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B736B4E-37A5-4EA1-A351-1AD78AE30906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C924FD93-5F50-4F91-8DED-5D5A2D0C7CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="問題マスター" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="297">
   <si>
     <t>id</t>
   </si>
@@ -458,9 +458,6 @@
   </si>
   <si>
     <t>択一の正解D</t>
-  </si>
-  <si>
-    <t>ks-001</t>
   </si>
   <si>
     <t>☆【2026年】(JPN)新規機械部門学科試験問題集_真偽法</t>
@@ -1488,13 +1485,172 @@
   </si>
   <si>
     <t>管理, PDCA, Plan, Do, Check, Action, スパイラルアップ</t>
+  </si>
+  <si>
+    <t>imageFile</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>explanationImageFile</t>
+  </si>
+  <si>
+    <t>id</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>ks-001</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>i-ks-502.png</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>i-kt-041.png</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>ks-502</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>kt-041</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Carlito"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>☆</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>【</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>年】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(JPN)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>新規機械部門学科試験問題集</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>択一試験用</t>
+    </r>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>☆【2026年】(JPN)新規機械部門学科試験問題集_択一試験用</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>測定・品質・製図規格</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>安全衛生・法令・その他</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>力Pの分力(P1,P2)は、図Bが正しい。</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>日本工業規格(JIS)による名称と記号の組合せとして、誤っているものはどれか。</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>A</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>B</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>C</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>D</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>力を2つの分力に分解する場合、元の力Pは平行四辺形の対角線になり、P₁・P₂はその隣り合う2辺になる。図BではP₁・P₂の合力がPと同じ向きの対角線になっていないため、正しい分力図ではない。</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>シャトル弁 — 2つの入力のうち圧力の高い側を出口へ導く弁の記号で、組合せは正しい。</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>逆止め弁（ばね付き） — ばねで弁を閉じ、順方向だけ流して逆流を止める記号で、組合せは正しい。</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>リリーフ弁 — 設定圧を超えた油を逃がして回路圧を制限する圧力制御弁の記号で、組合せは正しい。</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>減圧弁 — 図の記号は減圧弁ではなく絞り弁・可変絞り弁を表すため、組合せは誤り。</t>
+    <phoneticPr fontId="4"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1570,6 +1726,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="6"/>
+      <name val="Carlito"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1607,7 +1769,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1639,6 +1801,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1806,7 +1971,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y16"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr defaultRowHeight="8.4"/>
   <cols>
     <col min="1" max="1" width="9" style="9" bestFit="1" customWidth="1"/>
@@ -1817,23 +1982,24 @@
     <col min="6" max="6" width="7.296875" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.796875" style="9" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="35.59765625" style="10" customWidth="1"/>
-    <col min="9" max="12" width="26.796875" style="10" customWidth="1"/>
-    <col min="13" max="16" width="34" style="9" customWidth="1"/>
-    <col min="17" max="17" width="4.8984375" style="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="34" style="9" customWidth="1"/>
-    <col min="19" max="19" width="8.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.296875" style="9" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.59765625" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.796875" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="13" width="26.796875" style="10" customWidth="1"/>
+    <col min="14" max="17" width="34" style="9" customWidth="1"/>
+    <col min="18" max="18" width="4.8984375" style="9" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="34" style="9" customWidth="1"/>
+    <col min="21" max="21" width="8.5" style="9" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="5.296875" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.69921875" style="9" customWidth="1"/>
-    <col min="26" max="16384" width="8.796875" style="9"/>
+    <col min="23" max="23" width="7.59765625" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5" style="9" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="7" style="9" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.69921875" style="9" customWidth="1"/>
+    <col min="28" max="16384" width="8.796875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1">
+    <row r="1" spans="1:27" ht="24" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>0</v>
+        <v>276</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
@@ -1857,63 +2023,69 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="P1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="R1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="S1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="T1" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="U1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="V1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="W1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="X1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="Y1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="16.8">
+    <row r="2" spans="1:27" ht="16.8">
       <c r="A2" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>145</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>146</v>
       </c>
       <c r="C2" s="9">
         <v>1</v>
@@ -1922,48 +2094,48 @@
         <v>123</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F2" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>251</v>
-      </c>
       <c r="H2" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="Q2" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R2" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="S2" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T2" s="9" t="s">
-        <v>127</v>
+        <v>187</v>
+      </c>
+      <c r="R2" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S2" s="9" t="s">
+        <v>220</v>
       </c>
       <c r="U2" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V2" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W2" s="9">
-        <v>1</v>
-      </c>
-      <c r="X2" s="11">
+      <c r="V2" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="W2" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X2" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="16.8">
+    <row r="3" spans="1:27" ht="16.8">
       <c r="A3" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C3" s="9">
         <v>2</v>
@@ -1972,48 +2144,48 @@
         <v>123</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="Q3" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R3" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="S3" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" s="9" t="s">
-        <v>27</v>
+        <v>188</v>
+      </c>
+      <c r="R3" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>221</v>
       </c>
       <c r="U3" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V3" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W3" s="9">
-        <v>1</v>
-      </c>
-      <c r="X3" s="11">
+      <c r="V3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="W3" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X3" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="16.8">
+    <row r="4" spans="1:27" ht="16.8">
       <c r="A4" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C4" s="9">
         <v>3</v>
@@ -2022,48 +2194,48 @@
         <v>123</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q4" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R4" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="S4" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T4" s="9" t="s">
-        <v>139</v>
+        <v>189</v>
+      </c>
+      <c r="R4" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S4" s="9" t="s">
+        <v>222</v>
       </c>
       <c r="U4" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V4" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W4" s="9">
-        <v>1</v>
-      </c>
-      <c r="X4" s="11">
+      <c r="V4" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="W4" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X4" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="16.8">
+    <row r="5" spans="1:27" ht="16.8">
       <c r="A5" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C5" s="9">
         <v>4</v>
@@ -2072,48 +2244,48 @@
         <v>123</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F5" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="G5" s="9" t="s">
-        <v>255</v>
-      </c>
       <c r="H5" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q5" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R5" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="S5" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T5" s="9" t="s">
-        <v>127</v>
+        <v>190</v>
+      </c>
+      <c r="R5" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S5" s="9" t="s">
+        <v>223</v>
       </c>
       <c r="U5" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V5" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W5" s="9">
-        <v>1</v>
-      </c>
-      <c r="X5" s="11">
+      <c r="V5" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="W5" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X5" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="16.8">
+    <row r="6" spans="1:27" ht="16.8">
       <c r="A6" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C6" s="9">
         <v>5</v>
@@ -2122,48 +2294,48 @@
         <v>123</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q6" s="9" t="b">
+        <v>191</v>
+      </c>
+      <c r="R6" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="R6" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="S6" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T6" s="9" t="s">
-        <v>27</v>
+      <c r="S6" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="U6" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V6" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W6" s="9">
-        <v>1</v>
-      </c>
-      <c r="X6" s="11">
+      <c r="V6" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="W6" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X6" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="25.2">
+    <row r="7" spans="1:27" ht="27">
       <c r="A7" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>282</v>
       </c>
       <c r="C7" s="9">
         <v>1</v>
@@ -2172,69 +2344,69 @@
         <v>25</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F7" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>258</v>
-      </c>
       <c r="H7" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="I7" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="K7" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="L7" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="K7" s="10" t="s">
+      <c r="M7" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="L7" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="M7" s="9" t="s">
+      <c r="N7" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="O7" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="N7" s="9" t="s">
+      <c r="P7" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q7" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="O7" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="P7" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="Q7" s="9" t="s">
+      <c r="R7" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="S7" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T7" s="9" t="s">
+      <c r="U7" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V7" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="U7" s="9" t="b">
+      <c r="W7" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V7" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W7" s="9">
-        <v>1</v>
-      </c>
-      <c r="X7" s="11">
+      <c r="X7" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="25.2">
+    <row r="8" spans="1:27" ht="25.2">
       <c r="A8" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C8" s="9">
         <v>2</v>
@@ -2243,69 +2415,69 @@
         <v>25</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F8" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="G8" s="9" t="s">
-        <v>260</v>
-      </c>
       <c r="H8" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="I8" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="L8" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="M8" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="L8" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="M8" s="9" t="s">
+      <c r="N8" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="O8" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="N8" s="9" t="s">
+      <c r="P8" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q8" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="O8" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="P8" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="Q8" s="9" t="s">
+      <c r="R8" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="S8" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T8" s="9" t="s">
+      <c r="U8" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V8" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="U8" s="9" t="b">
+      <c r="W8" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V8" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W8" s="9">
-        <v>1</v>
-      </c>
-      <c r="X8" s="11">
+      <c r="X8" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="25.2">
+    <row r="9" spans="1:27" ht="25.2">
       <c r="A9" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C9" s="9">
         <v>3</v>
@@ -2314,69 +2486,69 @@
         <v>25</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="I9" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="M9" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="L9" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="M9" s="9" t="s">
+      <c r="N9" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="O9" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="N9" s="9" t="s">
+      <c r="P9" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="O9" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>232</v>
-      </c>
       <c r="Q9" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="R9" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="S9" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" s="9" t="s">
+      <c r="U9" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="U9" s="9" t="b">
+      <c r="W9" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V9" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W9" s="9">
-        <v>1</v>
-      </c>
-      <c r="X9" s="11">
+      <c r="X9" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z9" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="25.2">
+    <row r="10" spans="1:27" ht="25.2">
       <c r="A10" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C10" s="9">
         <v>4</v>
@@ -2385,69 +2557,69 @@
         <v>25</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F10" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="G10" s="9" t="s">
-        <v>263</v>
-      </c>
       <c r="H10" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="I10" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="L10" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="K10" s="10" t="s">
+      <c r="M10" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="L10" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="M10" s="9" t="s">
+      <c r="N10" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="O10" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="N10" s="9" t="s">
+      <c r="P10" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="O10" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="P10" s="9" t="s">
-        <v>233</v>
-      </c>
       <c r="Q10" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="R10" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="S10" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T10" s="9" t="s">
+      <c r="U10" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V10" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="U10" s="9" t="b">
+      <c r="W10" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V10" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W10" s="9">
-        <v>1</v>
-      </c>
-      <c r="X10" s="11">
+      <c r="X10" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="25.2">
+    <row r="11" spans="1:27" ht="25.2">
       <c r="A11" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C11" s="9">
         <v>5</v>
@@ -2456,69 +2628,69 @@
         <v>25</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="I11" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="K11" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="L11" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="K11" s="10" t="s">
+      <c r="M11" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="L11" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="M11" s="9" t="s">
-        <v>234</v>
-      </c>
       <c r="N11" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="O11" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="P11" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="O11" s="9" t="s">
+      <c r="Q11" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="P11" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="Q11" s="9" t="s">
+      <c r="R11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="S11" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T11" s="9" t="s">
+      <c r="U11" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V11" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="U11" s="9" t="b">
+      <c r="W11" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V11" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W11" s="9">
-        <v>1</v>
-      </c>
-      <c r="X11" s="11">
+      <c r="X11" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="26.4">
+    <row r="12" spans="1:27" ht="26.4">
       <c r="A12" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>157</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>158</v>
       </c>
       <c r="C12" s="9">
         <v>1</v>
@@ -2527,48 +2699,50 @@
         <v>123</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F12" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="G12" s="9" t="s">
-        <v>266</v>
-      </c>
       <c r="H12" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="I12" s="12"/>
+      <c r="R12" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S12" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="Q12" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R12" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="S12" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T12" s="9" t="s">
-        <v>27</v>
-      </c>
+      <c r="T12" s="13"/>
       <c r="U12" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V12" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W12" s="9">
-        <v>1</v>
-      </c>
-      <c r="X12" s="11">
+      <c r="V12" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X12" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y12" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="33.6">
+    <row r="13" spans="1:27" ht="33.6">
       <c r="A13" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C13" s="9">
         <v>2</v>
@@ -2577,48 +2751,49 @@
         <v>123</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F13" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>268</v>
-      </c>
       <c r="H13" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q13" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R13" s="14" t="s">
-        <v>200</v>
-      </c>
-      <c r="S13" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T13" s="9" t="s">
-        <v>139</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="R13" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="T13" s="14"/>
       <c r="U13" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V13" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W13" s="9">
-        <v>1</v>
-      </c>
-      <c r="X13" s="11">
+      <c r="V13" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="W13" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X13" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z13" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="25.2">
+    <row r="14" spans="1:27" ht="25.2">
       <c r="A14" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C14" s="9">
         <v>3</v>
@@ -2627,48 +2802,48 @@
         <v>123</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F14" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="G14" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>270</v>
-      </c>
       <c r="H14" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="Q14" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R14" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="S14" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T14" s="9" t="s">
-        <v>127</v>
+        <v>176</v>
+      </c>
+      <c r="R14" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" s="9" t="s">
+        <v>178</v>
       </c>
       <c r="U14" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V14" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W14" s="9">
-        <v>1</v>
-      </c>
-      <c r="X14" s="11">
+      <c r="V14" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="W14" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X14" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="25.2">
+    <row r="15" spans="1:27" ht="25.2">
       <c r="A15" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C15" s="9">
         <v>4</v>
@@ -2677,48 +2852,48 @@
         <v>123</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F15" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G15" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="G15" s="9" t="s">
-        <v>272</v>
-      </c>
       <c r="H15" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q15" s="9" t="b">
+        <v>180</v>
+      </c>
+      <c r="R15" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="R15" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="S15" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T15" s="9" t="s">
-        <v>27</v>
+      <c r="S15" s="9" t="s">
+        <v>182</v>
       </c>
       <c r="U15" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V15" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W15" s="9">
-        <v>1</v>
-      </c>
-      <c r="X15" s="11">
+      <c r="V15" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="W15" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X15" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z15" s="11">
         <v>46209</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="16.8">
+    <row r="16" spans="1:27" ht="16.8">
       <c r="A16" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C16" s="9">
         <v>5</v>
@@ -2727,40 +2902,155 @@
         <v>123</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F16" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="G16" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>274</v>
-      </c>
       <c r="H16" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="Q16" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R16" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="S16" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T16" s="9" t="s">
-        <v>139</v>
+        <v>184</v>
+      </c>
+      <c r="R16" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S16" s="9" t="s">
+        <v>186</v>
       </c>
       <c r="U16" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="V16" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="W16" s="9">
-        <v>1</v>
-      </c>
-      <c r="X16" s="11">
+      <c r="V16" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="W16" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X16" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y16" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z16" s="11">
         <v>46209</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" ht="16.8">
+      <c r="A17" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C17" s="9">
+        <v>502</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="R17" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="S17" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="U17" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="V17" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="W17" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X17" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y17" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z17" s="11">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" ht="25.2">
+      <c r="A18" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="C18" s="9">
+        <v>41</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="N18" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="O18" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="P18" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q18" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="R18" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="U18" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="V18" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="W18" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="X18" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y18" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z18" s="11">
+        <v>46210</v>
       </c>
     </row>
   </sheetData>
@@ -2769,13 +3059,13 @@
     <dataValidation type="list" sqref="D2:D999" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"true_false,multiple_choice"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:Q999" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="R2:R999" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"TRUE,FALSE,A,B,C,D"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="U2:V999 S2:S999" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" sqref="W2:X999 U2:U999" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="T2:T999" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" sqref="V2:V999" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"easy,normal,hard"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2790,302 +3080,302 @@
   <sheetData>
     <row r="2" spans="2:3">
       <c r="B2" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="2:3">
       <c r="C7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="2:3">
       <c r="B11" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="2:3">
       <c r="B12" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="2:3">
       <c r="B13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="2:3">
       <c r="B15" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="2:3">
       <c r="B16" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="17" spans="2:22">
       <c r="B17" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="2:22">
       <c r="B18" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19" spans="2:22">
       <c r="B19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="2:22">
       <c r="B21" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="2:22">
       <c r="B22" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" spans="2:22">
       <c r="B23" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" spans="2:22">
       <c r="B31" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="S31" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="T31" t="s">
         <v>226</v>
       </c>
-      <c r="S31" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="T31" t="s">
+      <c r="U31" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="V31" t="s">
         <v>227</v>
-      </c>
-      <c r="U31" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="V31" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="32" spans="2:22">
       <c r="B32" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="33" spans="2:22">
       <c r="B33" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="34" spans="2:22">
       <c r="B34" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="37" spans="2:22">
       <c r="B37" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="38" spans="2:22">
       <c r="B38" t="s">
+        <v>229</v>
+      </c>
+      <c r="S38" t="s">
+        <v>228</v>
+      </c>
+      <c r="T38" t="s">
+        <v>229</v>
+      </c>
+      <c r="U38" t="s">
+        <v>235</v>
+      </c>
+      <c r="V38" t="s">
         <v>230</v>
-      </c>
-      <c r="S38" t="s">
-        <v>229</v>
-      </c>
-      <c r="T38" t="s">
-        <v>230</v>
-      </c>
-      <c r="U38" t="s">
-        <v>236</v>
-      </c>
-      <c r="V38" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="39" spans="2:22">
       <c r="B39" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="40" spans="2:22">
       <c r="B40" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="43" spans="2:22">
       <c r="B43" t="s">
+        <v>236</v>
+      </c>
+      <c r="S43" t="s">
+        <v>236</v>
+      </c>
+      <c r="T43" t="s">
         <v>237</v>
       </c>
-      <c r="S43" t="s">
-        <v>237</v>
-      </c>
-      <c r="T43" t="s">
+      <c r="U43" t="s">
         <v>238</v>
       </c>
-      <c r="U43" t="s">
-        <v>239</v>
-      </c>
       <c r="V43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="44" spans="2:22">
       <c r="B44" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="45" spans="2:22">
       <c r="B45" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="46" spans="2:22">
       <c r="B46" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="51" spans="2:22">
       <c r="B51" t="s">
+        <v>239</v>
+      </c>
+      <c r="S51" t="s">
+        <v>239</v>
+      </c>
+      <c r="T51" t="s">
         <v>240</v>
       </c>
-      <c r="S51" t="s">
-        <v>240</v>
-      </c>
-      <c r="T51" t="s">
+      <c r="U51" t="s">
         <v>241</v>
       </c>
-      <c r="U51" t="s">
-        <v>242</v>
-      </c>
       <c r="V51" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="52" spans="2:22">
       <c r="B52" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="53" spans="2:22">
       <c r="B53" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="54" spans="2:22">
       <c r="B54" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="57" spans="2:22">
       <c r="B57" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S57" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="T57" t="s">
+        <v>242</v>
+      </c>
+      <c r="U57" t="s">
         <v>243</v>
       </c>
-      <c r="U57" t="s">
+      <c r="V57" t="s">
         <v>244</v>
-      </c>
-      <c r="V57" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="58" spans="2:22">
       <c r="B58" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="59" spans="2:22">
       <c r="B59" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="60" spans="2:22">
       <c r="B60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="68" spans="2:2">
       <c r="B68" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="69" spans="2:2">
       <c r="B69" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="70" spans="2:2">
       <c r="B70" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="71" spans="2:2">
       <c r="B71" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="72" spans="2:2">
       <c r="B72" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="76" spans="2:2">
       <c r="B76" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="77" spans="2:2">
       <c r="B77" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="78" spans="2:2">
       <c r="B78" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="79" spans="2:2">
       <c r="B79" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="80" spans="2:2">
       <c r="B80" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Switch JSON generation to full question master
</commit_message>
<xml_diff>
--- a/data/question_master_test_1.xlsx
+++ b/data/question_master_test_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\km78617\Documents\GitHub\kikai-gakka-exam\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C924FD93-5F50-4F91-8DED-5D5A2D0C7CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24DFC849-3867-4D0A-A48C-6878B5DE8A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1415,9 +1415,6 @@
     <t>ドリル・穴あけ</t>
   </si>
   <si>
-    <t>ステンレス鋼, 窒化鋼, 被削性, ドリル, 先端角</t>
-  </si>
-  <si>
     <t>穴あけ, ドリル, チゼル角, 食付き, 多角形</t>
   </si>
   <si>
@@ -1643,6 +1640,86 @@
   </si>
   <si>
     <t>減圧弁 — 図の記号は減圧弁ではなく絞り弁・可変絞り弁を表すため、組合せは誤り。</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ステンレス鋼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>窒化鋼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>被削性</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ドリル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>先端角</t>
+    </r>
     <phoneticPr fontId="4"/>
   </si>
 </sst>
@@ -1999,7 +2076,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="24" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
@@ -2023,7 +2100,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J1" s="7" t="s">
         <v>8</v>
@@ -2056,7 +2133,7 @@
         <v>17</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="U1" s="7" t="s">
         <v>18</v>
@@ -2082,7 +2159,7 @@
     </row>
     <row r="2" spans="1:27" ht="16.8">
       <c r="A2" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>145</v>
@@ -2099,8 +2176,8 @@
       <c r="F2" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>250</v>
+      <c r="G2" s="13" t="s">
+        <v>296</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>187</v>
@@ -2150,7 +2227,7 @@
         <v>249</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>188</v>
@@ -2200,7 +2277,7 @@
         <v>249</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>189</v>
@@ -2247,10 +2324,10 @@
         <v>247</v>
       </c>
       <c r="F5" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>253</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>254</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>190</v>
@@ -2297,10 +2374,10 @@
         <v>246</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>191</v>
@@ -2335,7 +2412,7 @@
         <v>150</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C7" s="9">
         <v>1</v>
@@ -2347,10 +2424,10 @@
         <v>246</v>
       </c>
       <c r="F7" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>257</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>192</v>
@@ -2418,10 +2495,10 @@
         <v>247</v>
       </c>
       <c r="F8" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>258</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>259</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>193</v>
@@ -2489,10 +2566,10 @@
         <v>247</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>194</v>
@@ -2560,10 +2637,10 @@
         <v>248</v>
       </c>
       <c r="F10" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>261</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>262</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>195</v>
@@ -2634,7 +2711,7 @@
         <v>249</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>196</v>
@@ -2702,10 +2779,10 @@
         <v>245</v>
       </c>
       <c r="F12" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>265</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>197</v>
@@ -2754,10 +2831,10 @@
         <v>245</v>
       </c>
       <c r="F13" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>266</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>267</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>167</v>
@@ -2805,10 +2882,10 @@
         <v>245</v>
       </c>
       <c r="F14" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="G14" s="9" t="s">
         <v>268</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>269</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>176</v>
@@ -2855,10 +2932,10 @@
         <v>245</v>
       </c>
       <c r="F15" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="G15" s="9" t="s">
         <v>270</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>271</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>180</v>
@@ -2905,10 +2982,10 @@
         <v>245</v>
       </c>
       <c r="F16" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="G16" s="9" t="s">
         <v>272</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>273</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>184</v>
@@ -2940,7 +3017,7 @@
     </row>
     <row r="17" spans="1:26" ht="16.8">
       <c r="A17" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>145</v>
@@ -2952,19 +3029,19 @@
         <v>123</v>
       </c>
       <c r="E17" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="H17" s="10" t="s">
-        <v>286</v>
-      </c>
       <c r="I17" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="R17" s="9" t="b">
         <v>0</v>
       </c>
       <c r="S17" s="9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="U17" s="9" t="b">
         <v>0</v>
@@ -2987,10 +3064,10 @@
     </row>
     <row r="18" spans="1:26" ht="25.2">
       <c r="A18" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C18" s="9">
         <v>41</v>
@@ -2999,37 +3076,37 @@
         <v>25</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H18" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="J18" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="I18" s="10" t="s">
-        <v>279</v>
-      </c>
-      <c r="J18" s="10" t="s">
+      <c r="K18" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="K18" s="10" t="s">
+      <c r="L18" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="L18" s="10" t="s">
+      <c r="M18" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="M18" s="10" t="s">
-        <v>291</v>
-      </c>
       <c r="N18" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="O18" s="9" t="s">
         <v>293</v>
       </c>
-      <c r="O18" s="9" t="s">
+      <c r="P18" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="P18" s="9" t="s">
+      <c r="Q18" s="9" t="s">
         <v>295</v>
-      </c>
-      <c r="Q18" s="9" t="s">
-        <v>296</v>
       </c>
       <c r="R18" s="9" t="s">
         <v>43</v>

</xml_diff>